<commit_message>
Test av redaktørleddet for dugnad 1 og 2: kildeinnboks lagt inn
- 41 nye kilder (K1201–K1241): digitaliseringsstrategien, NSM, SSB,
  KI-strategiinnspill 2019, NCSC, Nordlandsforskning, Arbeidstilsynet,
  Finanstilsynet, ekspertgruppen for KI og valg, Datatilsynet, Prop. 41 LS, Udir
- 62 tillegg i 42 temaer, 49 nye påstander, 19 «sjekk» besvart
- Dubletter slått sammen; K0271 fjernet som dublett
- Regler: privatpersoner i privat rolle, unntak fra 25-ordsgrensen for
  offentlige dokumenter, § 6 gjelder direkte uttalelser
- Sjekkpakker generert på nytt
</commit_message>
<xml_diff>
--- a/dugnad/sjekkpakker/DEM-03.xlsx
+++ b/dugnad/sjekkpakker/DEM-03.xlsx
@@ -172,7 +172,7 @@
     <t>Du kan bruke KI til å finne kilder, oppsummere og peke deg til rett sted i kilden. Men selve sjekken gjør du selv ved å lese originalen. Uten menneskelig verifisering er dugnaden verdiløs.</t>
   </si>
   <si>
-    <t>Privatpersoner navngis aldri.</t>
+    <t>Privatpersoner i privat rolle navngis aldri. Forskere og fagpersoner som uttaler seg offentlig i fagrollen sin, kan navngis.</t>
   </si>
   <si>
     <t>Spørsmål?</t>
@@ -406,7 +406,7 @@
     <t>[ukjent – bl.a. Finanstilsynet, Økokrim og journalistikk] – [Deepfakes av kjente nordmenn i falske investeringsannonser, og advarsler fra myndighetene]</t>
   </si>
   <si>
-    <t>Jo mer folk stoler på hverandre, desto mer lønner det seg å lure dem. Deepfakes av kjente nordmenn i falske investeringsannonser [K0699] (sjekk); svindeltall fra Finanstilsynet [K0185].</t>
+    <t>Jo mer folk stoler på hverandre, desto mer lønner det seg å lure dem. Deepfakes av kjente nordmenn i falske investeringsannonser [K0699] (sjekk); svindeltall fra Finanstilsynet [K0185] [K0262].</t>
   </si>
   <si>
     <t>ikke verifisert · Lagt til 2026-10-15 (DEM-03). Må finnes. · Eksistens (2026-10-25): usikker – Ingen Finanstilsynet-/Økokrim-varsel om navngitte nordmenn sett. Kandidater: Dagbladet om investeringssvindel med kjendiser og deepfake https://www.dagbladet.no/nyheter/utspekulert-svindel-nye-hver-uke/79113624 ; digi.no «Økokrim advarer om at næringslivet svindles ved hjelp av deepfake-teknologi» h</t>

</xml_diff>